<commit_message>
corrección coincidencias en PEPC
</commit_message>
<xml_diff>
--- a/Formato 3/precios_auxiliares_con_odoo.xlsx
+++ b/Formato 3/precios_auxiliares_con_odoo.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Auto-BT\Formato 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\Documents\Auto-BT\Formato 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5AD93A-EA68-48AF-AABC-A486E5684E95}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC10AE4-6221-45AD-93AD-C9600AA59B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="89">
   <si>
     <t>Código</t>
   </si>
@@ -209,6 +222,84 @@
   </si>
   <si>
     <t>P00707</t>
+  </si>
+  <si>
+    <t>IMC Diámetro 4"</t>
+  </si>
+  <si>
+    <t>P00049</t>
+  </si>
+  <si>
+    <t>IMC Diámetro 2"</t>
+  </si>
+  <si>
+    <t>P00048</t>
+  </si>
+  <si>
+    <t>IMC Diámetro 3/4"</t>
+  </si>
+  <si>
+    <t>P00046</t>
+  </si>
+  <si>
+    <t>TODO LÁMINAS C.E.</t>
+  </si>
+  <si>
+    <t>TMI (2) - 100 A- 10 kA - IP 44 - 600,700,250 - enero 2026</t>
+  </si>
+  <si>
+    <t>P00609</t>
+  </si>
+  <si>
+    <t>PROCABLES</t>
+  </si>
+  <si>
+    <t>Cable de cobre suave 12 AWG 600V THHN/THWN-2 PVC 90°C Seco</t>
+  </si>
+  <si>
+    <t>P00304</t>
+  </si>
+  <si>
+    <t>CENTELSA</t>
+  </si>
+  <si>
+    <t>Cable THHN/THWN-2 600V 8 AWG</t>
+  </si>
+  <si>
+    <t>P04028</t>
+  </si>
+  <si>
+    <t>Cables multiconductores de cobre MULTIFLEX 12 AWG 600V PVC/Nylon 90°C</t>
+  </si>
+  <si>
+    <t>P00288</t>
+  </si>
+  <si>
+    <t>TECNOWELD</t>
+  </si>
+  <si>
+    <t>SG1TN 6519</t>
+  </si>
+  <si>
+    <t>P00723</t>
+  </si>
+  <si>
+    <t>SG1TN 2694</t>
+  </si>
+  <si>
+    <t>P01244</t>
+  </si>
+  <si>
+    <t>LUHFSER</t>
+  </si>
+  <si>
+    <t>Tipo K de 65 Amperios para 15 kV - Frecuencia 50-60 Hz</t>
+  </si>
+  <si>
+    <t>P01386</t>
+  </si>
+  <si>
+    <t>ColmenaConduit</t>
   </si>
 </sst>
 </file>
@@ -311,9 +402,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -351,7 +442,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -457,7 +548,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -599,7 +690,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -607,13 +698,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="24.1796875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -627,7 +720,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -641,7 +734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -655,7 +748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -669,7 +762,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -683,7 +776,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -697,7 +790,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -711,7 +804,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -725,7 +818,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -739,7 +832,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -753,7 +846,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -767,7 +860,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
@@ -781,7 +874,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>35</v>
       </c>
@@ -795,7 +888,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -809,7 +902,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>41</v>
       </c>
@@ -823,7 +916,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>44</v>
       </c>
@@ -837,7 +930,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>47</v>
       </c>
@@ -851,7 +944,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>50</v>
       </c>
@@ -865,7 +958,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="58" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>53</v>
       </c>
@@ -879,7 +972,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>55</v>
       </c>
@@ -893,7 +986,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>56</v>
       </c>
@@ -907,7 +1000,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>57</v>
       </c>
@@ -919,6 +1012,160 @@
       </c>
       <c r="D22" s="1" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23">
+        <v>20000</v>
+      </c>
+      <c r="D23" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24">
+        <v>20000</v>
+      </c>
+      <c r="D24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25">
+        <v>1020000</v>
+      </c>
+      <c r="D25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26">
+        <v>183436.0410830999</v>
+      </c>
+      <c r="D26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27">
+        <v>133949.57983193299</v>
+      </c>
+      <c r="D27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>67</v>
+      </c>
+      <c r="B28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28">
+        <v>44285.714285714283</v>
+      </c>
+      <c r="D28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29">
+        <v>6467.8579103118018</v>
+      </c>
+      <c r="D29" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30">
+        <v>5840.3361344537816</v>
+      </c>
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31">
+        <v>9369.7478991596654</v>
+      </c>
+      <c r="D31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32">
+        <v>76211.000734891131</v>
+      </c>
+      <c r="D32" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" t="s">
+        <v>80</v>
+      </c>
+      <c r="C33">
+        <v>76211.000734891131</v>
+      </c>
+      <c r="D33" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>